<commit_message>
view detail chat WA & perbaikan format upload raw WA
</commit_message>
<xml_diff>
--- a/files/Format_Count_Response_Time_WA_GMT7.xlsx
+++ b/files/Format_Count_Response_Time_WA_GMT7.xlsx
@@ -205,7 +205,7 @@
     <t>6a1fa7a5235e9</t>
   </si>
   <si>
-    <t>Tantri</t>
+    <t>Dina</t>
   </si>
   <si>
     <t>agent</t>
@@ -308,8 +308,8 @@
   <numFmts count="5">
     <numFmt numFmtId="176" formatCode="dd\-mmm\-yyyy\ hh:mm:ss"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="178" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="21">
@@ -338,7 +338,114 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -353,98 +460,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -456,22 +472,6 @@
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="35">
     <fill>
@@ -500,55 +500,151 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -560,121 +656,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -716,16 +716,37 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4"/>
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -745,26 +766,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
+      <bottom style="medium">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -780,165 +786,159 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1351,7 +1351,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:P46"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.625" style="1"/>
@@ -2435,11 +2435,11 @@
     </row>
     <row r="22" spans="1:16">
       <c r="A22" s="5">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="A22:A46" si="2">DATE(LEFT(I22,4),MID(I22,6,2),MID(I22,9,2))+TIME(MID(I22,12,2)+7,MID(I22,15,2),MID(I22,18,2))</f>
         <v>46176.4959027778</v>
       </c>
       <c r="B22" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="B22:B46" si="3">IF(AND(H22="agent",H21="customer"),ROUND((A22-A21)*3600*24,0),"")</f>
         <v/>
       </c>
       <c r="C22" s="1" t="s">
@@ -2484,11 +2484,11 @@
     </row>
     <row r="23" spans="1:16">
       <c r="A23" s="5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>46176.4962847222</v>
       </c>
       <c r="B23" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="C23" s="1" t="s">
@@ -2532,6 +2532,236 @@
       </c>
       <c r="P23" s="1" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B24" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B25" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B26" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B27" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B28" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B29" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B30" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B31" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B32" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B33" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B34" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B35" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B36" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B37" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B38" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B39" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B40" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B41" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B42" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B43" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B44" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B45" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" s="5" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="B46" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>